<commit_message>
se implementa el indice
</commit_message>
<xml_diff>
--- a/errores.xlsx
+++ b/errores.xlsx
@@ -13,104 +13,10 @@
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 35 en PNT  </t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1033 en todo el pnt de control de calidad</t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1135 para el artículo PHB1V01. dentro de los articulos PHB1V01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 32 en PNT  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 36 en PNT  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 25 en PNT  </t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1137 para el artículo PHR1V01. dentro de los articulos PHR1V01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 26 en PNT  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 31 en PNT  </t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1033 para el artículo KITDCSDOMV03. dentro de los articulos KITDCSDOMV03</t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1135 en todo el pnt de control de calidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 22 en PNT  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 34 en PNT  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 27 en PNT  </t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1057 para el artículo KITDCSDOMV03. dentro de los articulos KITDCSDOMV03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 28 en PNT  </t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1057 en todo el pnt de control de calidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 21 en PNT  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 33 en PNT  </t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 921 para el artículo KITDCSDOMV03. dentro de los articulos KITDCSDOMV03</t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 921 en todo el pnt de control de calidad</t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 484 para el artículo PHR1V01. dentro de los articulos PHR1V01</t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 950 para el artículo KITDCSDOMV03. dentro de los articulos KITDCSDOMV03</t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 267 para el artículo PDV01. dentro de los articulos PDV01</t>
-  </si>
-  <si>
-    <t>No se encuentra el PNT de la orden 1137 en todo el pnt de control de calidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 29 en PNT  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">No se ha encontrado CMD4EPBV01 con lote 30 en PNT  </t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -126,7 +32,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -134,30 +40,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,150 +340,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1">
-      <c r="A14" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1">
-      <c r="A17" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1">
-      <c r="A22" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1">
-      <c r="A23" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1">
-      <c r="A24" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1">
-      <c r="A25" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1">
-      <c r="A26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1">
-      <c r="A27" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1">
-      <c r="A28" t="s">
-        <v>26</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se empieza la comprobacion de la informacion del bachrecord
</commit_message>
<xml_diff>
--- a/errores.xlsx
+++ b/errores.xlsx
@@ -13,10 +13,32 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+  <si>
+    <t>No se encuentra el PNT de la orden 1153 para el artículo EPTEV02DEV01. dentro de los articulos EPTEV02DEV01</t>
+  </si>
+  <si>
+    <t>No se encuentra el PNT de la orden 518 para el artículo EPTEV02DEV01. dentro de los articulos EPTEV02DEV01</t>
+  </si>
+  <si>
+    <t>No se encuentra el PNT de la orden 518 en todo el pnt de control de calidad</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -32,7 +54,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -40,12 +62,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -340,9 +380,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>